<commit_message>
Add transport_notes to resorts
`transport` answers which modes serve a resort, which is all the
Transportation Challenge needs — the badge is earned from what a user logs
riding, not from the catalog. It cannot answer "to where": the boat from
Wilderness Lodge and the boat from Beach Club go to different places, and the
same ambiguity applies to walk and monorail.

Nullable free text, added empty. Worth filling for the Crescent Lake walkers
and the Magic Kingdom walkway; pointless for a value resort whose only mode is
bus. Roughly a dozen rows, not all 34.

Also scopes the root tsconfig to exclude web/. The root include of **/*.tsx
was swallowing the Next app, whose tsconfig maps @/* to ./* rather than
./src/*, so every one of its imports failed to resolve. Broken since the site
was created; only surfaced now because web is typechecked by `next build`.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/catalog-entry.xlsx
+++ b/data/catalog-entry.xlsx
@@ -329,7 +329,13 @@
 a wrong value makes a badge unearnable.</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional, free text. What the modes actually connect to, e.g. "Walk or boat to EPCOT and Hollywood Studios".
+Fill only where it is not obvious. A value resort whose only mode is bus needs nothing here.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>THE GATE. Format YYYY-MM-DD.
 Rows without it are refused by
@@ -1890,7 +1896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1899,13 +1905,14 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1941,35 +1948,40 @@
       </c>
       <c r="G1" s="11" t="inlineStr">
         <is>
+          <t>transport_notes</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>lng</t>
         </is>
       </c>
-      <c r="I1" s="11" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>official_url</t>
         </is>
       </c>
-      <c r="J1" s="11" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="K1" s="11" t="inlineStr">
+      <c r="L1" s="11" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" s="11" t="inlineStr">
+      <c r="M1" s="11" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="M1" s="11" t="inlineStr">
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
@@ -2008,36 +2020,41 @@
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
+          <t>Monorail or boat to Magic Kingdom</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
           <t>28.405000</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="I2" s="10" t="inlineStr">
         <is>
           <t>-81.583000</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="J2" s="10" t="inlineStr">
         <is>
           <t>https://disneyworld.disney.go.com/resorts/polynesian-resort/</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="K2" s="10" t="inlineStr">
         <is>
           <t>Deluxe South Pacific themed resort on the monorail loop.</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="L2" s="10" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr"/>
       <c r="M2" s="10" t="inlineStr"/>
+      <c r="N2" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A3:M200">
+  <conditionalFormatting sqref="A3:N200">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
-      <formula>AND($A3&lt;&gt;"",$L3="")</formula>
+      <formula>AND($A3&lt;&gt;"",$M3="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
@@ -2050,7 +2067,7 @@
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Not a valid value. Pick from the dropdown." promptTitle="" type="list" errorStyle="stop">
       <formula1>=resort_tier</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Not a valid value. Pick from the dropdown." promptTitle="" type="list" errorStyle="stop">
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Not a valid value. Pick from the dropdown." promptTitle="" type="list" errorStyle="stop">
       <formula1>=status</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>